<commit_message>
Expand Data Modeling tab with Corewell-specific unified-model questions
Rework 8_Modeling from 10 generic questions to 33, grounded in this week's
discovery call: medallion layer semantics (Bronze/Silver/Gold/Share),
unified/conformed entity definitions, dbt Core modeling practices, semantic
layer consistency across Tableau/Power BI/Excel, and where PII/PHI masking
applies in the modeling layer. 18 questions flagged as directly tied to the
single-source-of-truth mandate from discovery.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gjis7Be5wDA62NCDragMb8
</commit_message>
<xml_diff>
--- a/Corewell_DDA_Questionnaire_v2.0.xlsx
+++ b/Corewell_DDA_Questionnaire_v2.0.xlsx
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -183,6 +183,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1085,18 +1088,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
@@ -1105,14 +1108,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>8. Data Modeling</t>
+          <t>8. Data Modeling  —  Unified Model / Single Source of Truth</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Corewell Snowflake DD&amp;A – capture Current State, Evidence, and Recommendation for each question. Score Maturity 1-5.</t>
+          <t>PRIMARY FOCUS DOMAIN per Corewell discovery (Jay, wk of Discovery). Highlighted rows tie directly to the unified-model / SSOT mandate. Ingestion &amp; Transformation domains are lower priority per client — tooling confirmed stable.</t>
         </is>
       </c>
     </row>
@@ -1178,42 +1181,42 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="9" t="n">
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="16" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Approach</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Modeling approach – Kimball star, Snowflake schema, Data Vault 2.0, 3NF, Wide table / OBT?</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" s="9" t="n"/>
-      <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
-      <c r="L5" s="9" t="n"/>
-    </row>
-    <row r="6" ht="38" customHeight="1">
+          <t>Medallion Layer Semantics</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Is there a documented layer contract for Bronze/Silver/Gold/Share — what belongs in each, ownership, and SLAs?</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="16" t="n"/>
+    </row>
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="9" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Approach</t>
+          <t>Medallion Layer Semantics</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Consistent modeling standards across domains?</t>
+          <t>Is Bronze strictly raw/immutable, or does any transformation happen before Silver?</t>
         </is>
       </c>
       <c r="D6" s="9" t="n"/>
@@ -1226,66 +1229,66 @@
       <c r="K6" s="9" t="n"/>
       <c r="L6" s="9" t="n"/>
     </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="9" t="n">
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="16" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Approach</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Conformed dimensions defined and reused?</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="9" t="n"/>
-      <c r="J7" s="9" t="n"/>
-      <c r="K7" s="9" t="n"/>
-      <c r="L7" s="9" t="n"/>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="9" t="n">
+          <t>Medallion Layer Semantics</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>What formally differentiates Gold from Share — is Share a governed export/exposure layer, or a duplicate of Gold for external consumers?</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="16" t="n"/>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="16" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Techniques</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Slowly Changing Dimensions – which types (1/2/3/6) and where?</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
-      <c r="L8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="38" customHeight="1">
+          <t>Medallion Layer Semantics</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Do any BI tools (Tableau, Power BI, Excel) read directly from Silver or Bronze, bypassing Gold?</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="16" t="n"/>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="16" t="n"/>
+      <c r="H8" s="16" t="n"/>
+      <c r="I8" s="16" t="n"/>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="16" t="n"/>
+      <c r="L8" s="16" t="n"/>
+    </row>
+    <row r="9" ht="40" customHeight="1">
       <c r="A9" s="9" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Techniques</t>
+          <t>Medallion Layer Semantics</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Fact table grain documented per fact?</t>
+          <t>Is there a formal promotion process (Silver → Gold) with data quality gates before promotion?</t>
         </is>
       </c>
       <c r="D9" s="9" t="n"/>
@@ -1298,18 +1301,18 @@
       <c r="K9" s="9" t="n"/>
       <c r="L9" s="9" t="n"/>
     </row>
-    <row r="10" ht="38" customHeight="1">
+    <row r="10" ht="40" customHeight="1">
       <c r="A10" s="9" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Techniques</t>
+          <t>Medallion Layer Semantics</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Materialized Views used – where and why?</t>
+          <t>Is the Share layer partitioned/scoped by consumer (per team, per external partner), or is it one shared export?</t>
         </is>
       </c>
       <c r="D10" s="9" t="n"/>
@@ -1322,101 +1325,653 @@
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
     </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="9" t="n">
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="16" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Techniques</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Dynamic Tables in use? Refresh lag configured?</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="9" t="n"/>
-      <c r="I11" s="9" t="n"/>
-      <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n"/>
-      <c r="L11" s="9" t="n"/>
-    </row>
-    <row r="12" ht="38" customHeight="1">
-      <c r="A12" s="9" t="n">
+          <t>Unified Data Model / Single Source of Truth</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Is there a canonical, conformed definition for core business entities (e.g. Patient, Provider, Encounter, Facility, Claim)? Where is it documented?</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="16" t="n"/>
+      <c r="H11" s="16" t="n"/>
+      <c r="I11" s="16" t="n"/>
+      <c r="J11" s="16" t="n"/>
+      <c r="K11" s="16" t="n"/>
+      <c r="L11" s="16" t="n"/>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="16" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Techniques</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Views vs Tables strategy for consumption layer?</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n"/>
-      <c r="J12" s="9" t="n"/>
-      <c r="K12" s="9" t="n"/>
-      <c r="L12" s="9" t="n"/>
-    </row>
-    <row r="13" ht="38" customHeight="1">
-      <c r="A13" s="9" t="n">
+          <t>Unified Data Model / Single Source of Truth</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>How are conflicting definitions of the same entity across domains (e.g. "active patient," "current provider") reconciled today?</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="n"/>
+      <c r="E12" s="16" t="n"/>
+      <c r="F12" s="16" t="n"/>
+      <c r="G12" s="16" t="n"/>
+      <c r="H12" s="16" t="n"/>
+      <c r="I12" s="16" t="n"/>
+      <c r="J12" s="16" t="n"/>
+      <c r="K12" s="16" t="n"/>
+      <c r="L12" s="16" t="n"/>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="16" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Semantic Layer</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Is there a semantic layer (dbt semantic layer / Cube / AtScale / BI-native)?</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n"/>
-      <c r="I13" s="9" t="n"/>
-      <c r="J13" s="9" t="n"/>
-      <c r="K13" s="9" t="n"/>
-      <c r="L13" s="9" t="n"/>
-    </row>
-    <row r="14" ht="38" customHeight="1">
-      <c r="A14" s="9" t="n">
+          <t>Unified Data Model / Single Source of Truth</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>How many parallel "sources of truth" currently exist for the same core entities across Gold models?</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="16" t="n"/>
+      <c r="F13" s="16" t="n"/>
+      <c r="G13" s="16" t="n"/>
+      <c r="H13" s="16" t="n"/>
+      <c r="I13" s="16" t="n"/>
+      <c r="J13" s="16" t="n"/>
+      <c r="K13" s="16" t="n"/>
+      <c r="L13" s="16" t="n"/>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="16" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Semantic Layer</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Metric definitions centralized to avoid duplication in Tableau / PowerBI / SAS?</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="n"/>
-      <c r="J14" s="9" t="n"/>
-      <c r="K14" s="9" t="n"/>
-      <c r="L14" s="9" t="n"/>
+          <t>Unified Data Model / Single Source of Truth</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Is there a Master Data Management (MDM) capability or golden-record process for key entities?</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="16" t="n"/>
+      <c r="F14" s="16" t="n"/>
+      <c r="G14" s="16" t="n"/>
+      <c r="H14" s="16" t="n"/>
+      <c r="I14" s="16" t="n"/>
+      <c r="J14" s="16" t="n"/>
+      <c r="K14" s="16" t="n"/>
+      <c r="L14" s="16" t="n"/>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Unified Data Model / Single Source of Truth</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Who owns the enterprise conceptual/logical data model, if one exists?</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="16" t="n"/>
+      <c r="F15" s="16" t="n"/>
+      <c r="G15" s="16" t="n"/>
+      <c r="H15" s="16" t="n"/>
+      <c r="I15" s="16" t="n"/>
+      <c r="J15" s="16" t="n"/>
+      <c r="K15" s="16" t="n"/>
+      <c r="L15" s="16" t="n"/>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Unified Data Model / Single Source of Truth</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Is there an entity-relationship diagram or data dictionary covering the Gold layer?</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="9" t="n"/>
+      <c r="L16" s="9" t="n"/>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Unified Data Model / Single Source of Truth</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Is there a process for onboarding a new domain's data into the unified model, or does each domain model independently today?</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="n"/>
+      <c r="G17" s="16" t="n"/>
+      <c r="H17" s="16" t="n"/>
+      <c r="I17" s="16" t="n"/>
+      <c r="J17" s="16" t="n"/>
+      <c r="K17" s="16" t="n"/>
+      <c r="L17" s="16" t="n"/>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Modeling Standards &amp; Approach</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>What modeling pattern is used in Gold — Kimball star schema, Data Vault, One Big Table, 3NF, or ad hoc per team?</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="9" t="n"/>
+      <c r="F18" s="9" t="n"/>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
+      <c r="I18" s="9" t="n"/>
+      <c r="J18" s="9" t="n"/>
+      <c r="K18" s="9" t="n"/>
+      <c r="L18" s="9" t="n"/>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Modeling Standards &amp; Approach</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Is the modeling approach consistent across domains, or does each team choose independently?</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="n"/>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="16" t="n"/>
+      <c r="I19" s="16" t="n"/>
+      <c r="J19" s="16" t="n"/>
+      <c r="K19" s="16" t="n"/>
+      <c r="L19" s="16" t="n"/>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Modeling Standards &amp; Approach</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Are conformed dimensions (Date, Patient, Provider, Facility) shared and reused across fact tables, or duplicated per domain?</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="n"/>
+      <c r="G20" s="16" t="n"/>
+      <c r="H20" s="16" t="n"/>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="16" t="n"/>
+      <c r="K20" s="16" t="n"/>
+      <c r="L20" s="16" t="n"/>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Modeling Standards &amp; Approach</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Is fact table grain documented and enforced per fact table?</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="9" t="n"/>
+      <c r="G21" s="9" t="n"/>
+      <c r="H21" s="9" t="n"/>
+      <c r="I21" s="9" t="n"/>
+      <c r="J21" s="9" t="n"/>
+      <c r="K21" s="9" t="n"/>
+      <c r="L21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Modeling Standards &amp; Approach</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Which Slowly Changing Dimension types (1/2/3/6) are used, and is history tracked consistently across domains?</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>dbt Core Modeling Practices</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>How are dbt models organized (staging / intermediate / marts), and how does that map to Bronze/Silver/Gold/Share?</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
+      <c r="J23" s="9" t="n"/>
+      <c r="K23" s="9" t="n"/>
+      <c r="L23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>dbt Core Modeling Practices</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Are naming conventions for models, sources, and columns documented and enforced in dbt?</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n"/>
+      <c r="I24" s="9" t="n"/>
+      <c r="J24" s="9" t="n"/>
+      <c r="K24" s="9" t="n"/>
+      <c r="L24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>dbt Core Modeling Practices</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Are dbt tests (uniqueness, not-null, relationships, custom) applied consistently across Gold models?</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n"/>
+      <c r="I25" s="9" t="n"/>
+      <c r="J25" s="9" t="n"/>
+      <c r="K25" s="9" t="n"/>
+      <c r="L25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>dbt Core Modeling Practices</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Is dbt docs / the lineage DAG kept current and used for model discovery?</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="9" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="9" t="n"/>
+      <c r="L26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>dbt Core Modeling Practices</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Are dbt exposures used to track which Tableau/Power BI/Excel reports depend on which models?</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="16" t="n"/>
+      <c r="F27" s="16" t="n"/>
+      <c r="G27" s="16" t="n"/>
+      <c r="H27" s="16" t="n"/>
+      <c r="I27" s="16" t="n"/>
+      <c r="J27" s="16" t="n"/>
+      <c r="K27" s="16" t="n"/>
+      <c r="L27" s="16" t="n"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>dbt Core Modeling Practices</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>How is modeling technical debt tracked today (deprecated models, workaround joins, known hacks)?</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="16" t="n"/>
+      <c r="G28" s="16" t="n"/>
+      <c r="H28" s="16" t="n"/>
+      <c r="I28" s="16" t="n"/>
+      <c r="J28" s="16" t="n"/>
+      <c r="K28" s="16" t="n"/>
+      <c r="L28" s="16" t="n"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Semantic Layer &amp; BI Consumption</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Is there a shared semantic/metrics layer, or does each BI tool (Tableau, Power BI, Excel) define its own metrics independently?</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="16" t="n"/>
+      <c r="G29" s="16" t="n"/>
+      <c r="H29" s="16" t="n"/>
+      <c r="I29" s="16" t="n"/>
+      <c r="J29" s="16" t="n"/>
+      <c r="K29" s="16" t="n"/>
+      <c r="L29" s="16" t="n"/>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Semantic Layer &amp; BI Consumption</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>How much metric duplication or inconsistency exists across Tableau vs. Power BI vs. Excel reports today for the same KPI?</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="n"/>
+      <c r="E30" s="16" t="n"/>
+      <c r="F30" s="16" t="n"/>
+      <c r="G30" s="16" t="n"/>
+      <c r="H30" s="16" t="n"/>
+      <c r="I30" s="16" t="n"/>
+      <c r="J30" s="16" t="n"/>
+      <c r="K30" s="16" t="n"/>
+      <c r="L30" s="16" t="n"/>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Semantic Layer &amp; BI Consumption</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>How is business logic embedded in Tableau/Power BI calculated fields reconciled with logic already in the dbt/Gold layer (logic leakage)?</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="16" t="n"/>
+      <c r="F31" s="16" t="n"/>
+      <c r="G31" s="16" t="n"/>
+      <c r="H31" s="16" t="n"/>
+      <c r="I31" s="16" t="n"/>
+      <c r="J31" s="16" t="n"/>
+      <c r="K31" s="16" t="n"/>
+      <c r="L31" s="16" t="n"/>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Semantic Layer &amp; BI Consumption</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>What is the process for evolving or versioning a Gold model without breaking downstream Tableau/Power BI/Excel consumers?</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="9" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n"/>
+      <c r="I32" s="9" t="n"/>
+      <c r="J32" s="9" t="n"/>
+      <c r="K32" s="9" t="n"/>
+      <c r="L32" s="9" t="n"/>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Governance &amp; Sensitive Data in the Model</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>Where are PII/PHI attributes identified and tagged within the modeling layer — at Bronze, Silver, or only at Gold/Share?</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="n"/>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="16" t="n"/>
+      <c r="G33" s="16" t="n"/>
+      <c r="H33" s="16" t="n"/>
+      <c r="I33" s="16" t="n"/>
+      <c r="J33" s="16" t="n"/>
+      <c r="K33" s="16" t="n"/>
+      <c r="L33" s="16" t="n"/>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="A34" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Governance &amp; Sensitive Data in the Model</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Are Row Access Policies (RLS) or Column-level masking (CLS) applied at the Gold/Share layer, or upstream in Silver?</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="n"/>
+      <c r="E34" s="16" t="n"/>
+      <c r="F34" s="16" t="n"/>
+      <c r="G34" s="16" t="n"/>
+      <c r="H34" s="16" t="n"/>
+      <c r="I34" s="16" t="n"/>
+      <c r="J34" s="16" t="n"/>
+      <c r="K34" s="16" t="n"/>
+      <c r="L34" s="16" t="n"/>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Governance &amp; Sensitive Data in the Model</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Is there a data classification standard applied consistently to modeled columns across all domains?</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="F35" s="9" t="n"/>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" s="9" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="9" t="n"/>
+      <c r="L35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="40" customHeight="1">
+      <c r="A36" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Governance &amp; Sensitive Data in the Model</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Who approves a new Gold/Share model before it's exposed to Tableau/Power BI/Excel?</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="9" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="9" t="n"/>
+      <c r="K36" s="9" t="n"/>
+      <c r="L36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Governance &amp; Sensitive Data in the Model</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Are data contracts in place between source-aligned teams and the modeling/analytics team for schema stability?</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="9" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
+      <c r="J37" s="9" t="n"/>
+      <c r="K37" s="9" t="n"/>
+      <c r="L37" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7188,13 +7743,13 @@
           <t>1. Organization &amp; Governance</t>
         </is>
       </c>
-      <c r="C5" s="12" t="str">
+      <c r="C5" s="12">
         <f>IFERROR(AVERAGE('1_Governance'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D5" s="9">
         <f>COUNT('1_Governance'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E5" s="9" t="n"/>
       <c r="F5" s="9" t="n"/>
@@ -7208,13 +7763,13 @@
           <t>2. Snowflake Account Architecture</t>
         </is>
       </c>
-      <c r="C6" s="12" t="str">
+      <c r="C6" s="12">
         <f>IFERROR(AVERAGE('2_AccountArch'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D6" s="9">
         <f>COUNT('2_AccountArch'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E6" s="9" t="n"/>
       <c r="F6" s="9" t="n"/>
@@ -7228,13 +7783,13 @@
           <t>3. Security &amp; Identity</t>
         </is>
       </c>
-      <c r="C7" s="12" t="str">
+      <c r="C7" s="12">
         <f>IFERROR(AVERAGE('3_Security'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D7" s="9">
         <f>COUNT('3_Security'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E7" s="9" t="n"/>
       <c r="F7" s="9" t="n"/>
@@ -7248,13 +7803,13 @@
           <t>4. Networking</t>
         </is>
       </c>
-      <c r="C8" s="12" t="str">
+      <c r="C8" s="12">
         <f>IFERROR(AVERAGE('4_Networking'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D8" s="9">
         <f>COUNT('4_Networking'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E8" s="9" t="n"/>
       <c r="F8" s="9" t="n"/>
@@ -7268,13 +7823,13 @@
           <t>5. Data Architecture</t>
         </is>
       </c>
-      <c r="C9" s="12" t="str">
+      <c r="C9" s="12">
         <f>IFERROR(AVERAGE('5_DataArch'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D9" s="9">
         <f>COUNT('5_DataArch'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E9" s="9" t="n"/>
       <c r="F9" s="9" t="n"/>
@@ -7288,13 +7843,13 @@
           <t>6. Data Ingestion</t>
         </is>
       </c>
-      <c r="C10" s="12" t="str">
+      <c r="C10" s="12">
         <f>IFERROR(AVERAGE('6_Ingestion'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D10" s="9">
         <f>COUNT('6_Ingestion'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E10" s="9" t="n"/>
       <c r="F10" s="9" t="n"/>
@@ -7308,13 +7863,13 @@
           <t>7. Data Transformation</t>
         </is>
       </c>
-      <c r="C11" s="12" t="str">
+      <c r="C11" s="12">
         <f>IFERROR(AVERAGE('7_Transform'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D11" s="9">
         <f>COUNT('7_Transform'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E11" s="9" t="n"/>
       <c r="F11" s="9" t="n"/>
@@ -7328,13 +7883,13 @@
           <t>8. Data Modeling</t>
         </is>
       </c>
-      <c r="C12" s="12" t="str">
+      <c r="C12" s="12">
         <f>IFERROR(AVERAGE('8_Modeling'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D12" s="9">
         <f>COUNT('8_Modeling'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E12" s="9" t="n"/>
       <c r="F12" s="9" t="n"/>
@@ -7348,13 +7903,13 @@
           <t>9. Compute &amp; Warehouses</t>
         </is>
       </c>
-      <c r="C13" s="12" t="str">
+      <c r="C13" s="12">
         <f>IFERROR(AVERAGE('9_Compute'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D13" s="9">
         <f>COUNT('9_Compute'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E13" s="9" t="n"/>
       <c r="F13" s="9" t="n"/>
@@ -7368,13 +7923,13 @@
           <t>10. Storage &amp; Data Lifecycle</t>
         </is>
       </c>
-      <c r="C14" s="12" t="str">
+      <c r="C14" s="12">
         <f>IFERROR(AVERAGE('10_Storage'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D14" s="9">
         <f>COUNT('10_Storage'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E14" s="9" t="n"/>
       <c r="F14" s="9" t="n"/>
@@ -7388,13 +7943,13 @@
           <t>11. Performance Optimization</t>
         </is>
       </c>
-      <c r="C15" s="12" t="str">
+      <c r="C15" s="12">
         <f>IFERROR(AVERAGE('11_Performance'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D15" s="9">
         <f>COUNT('11_Performance'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E15" s="9" t="n"/>
       <c r="F15" s="9" t="n"/>
@@ -7408,13 +7963,13 @@
           <t>12. Cost Optimization (FinOps)</t>
         </is>
       </c>
-      <c r="C16" s="12" t="str">
+      <c r="C16" s="12">
         <f>IFERROR(AVERAGE('12_FinOps'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D16" s="9">
         <f>COUNT('12_FinOps'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E16" s="9" t="n"/>
       <c r="F16" s="9" t="n"/>
@@ -7428,13 +7983,13 @@
           <t>13. Data Sharing &amp; Collaboration</t>
         </is>
       </c>
-      <c r="C17" s="12" t="str">
+      <c r="C17" s="12">
         <f>IFERROR(AVERAGE('13_Sharing'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D17" s="9">
         <f>COUNT('13_Sharing'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E17" s="9" t="n"/>
       <c r="F17" s="9" t="n"/>
@@ -7448,13 +8003,13 @@
           <t>14. Data Quality</t>
         </is>
       </c>
-      <c r="C18" s="12" t="str">
+      <c r="C18" s="12">
         <f>IFERROR(AVERAGE('14_DQ'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D18" s="9">
         <f>COUNT('14_DQ'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E18" s="9" t="n"/>
       <c r="F18" s="9" t="n"/>
@@ -7468,13 +8023,13 @@
           <t>15. Metadata &amp; Catalog</t>
         </is>
       </c>
-      <c r="C19" s="12" t="str">
+      <c r="C19" s="12">
         <f>IFERROR(AVERAGE('15_Metadata'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D19" s="9">
         <f>COUNT('15_Metadata'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E19" s="9" t="n"/>
       <c r="F19" s="9" t="n"/>
@@ -7488,13 +8043,13 @@
           <t>16. DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="C20" s="12" t="str">
+      <c r="C20" s="12">
         <f>IFERROR(AVERAGE('16_DevOps'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D20" s="9">
         <f>COUNT('16_DevOps'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E20" s="9" t="n"/>
       <c r="F20" s="9" t="n"/>
@@ -7508,13 +8063,13 @@
           <t>17. Monitoring &amp; Observability</t>
         </is>
       </c>
-      <c r="C21" s="12" t="str">
+      <c r="C21" s="12">
         <f>IFERROR(AVERAGE('17_Monitoring'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D21" s="9">
         <f>COUNT('17_Monitoring'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E21" s="9" t="n"/>
       <c r="F21" s="9" t="n"/>
@@ -7528,13 +8083,13 @@
           <t>18. Disaster Recovery &amp; BCP</t>
         </is>
       </c>
-      <c r="C22" s="12" t="str">
+      <c r="C22" s="12">
         <f>IFERROR(AVERAGE('18_DR'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D22" s="9">
         <f>COUNT('18_DR'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E22" s="9" t="n"/>
       <c r="F22" s="9" t="n"/>
@@ -7548,13 +8103,13 @@
           <t>19. AI / Cortex / ML Readiness</t>
         </is>
       </c>
-      <c r="C23" s="12" t="str">
+      <c r="C23" s="12">
         <f>IFERROR(AVERAGE('19_AI'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D23" s="9">
         <f>COUNT('19_AI'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="9" t="n"/>
@@ -7568,13 +8123,13 @@
           <t>20. Compliance &amp; Audit (HIPAA / HITRUST)</t>
         </is>
       </c>
-      <c r="C24" s="12" t="str">
+      <c r="C24" s="12">
         <f>IFERROR(AVERAGE('20_Compliance'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D24" s="9">
         <f>COUNT('20_Compliance'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E24" s="9" t="n"/>
       <c r="F24" s="9" t="n"/>
@@ -7588,13 +8143,13 @@
           <t>21. Operations &amp; SLA</t>
         </is>
       </c>
-      <c r="C25" s="12" t="str">
+      <c r="C25" s="12">
         <f>IFERROR(AVERAGE('21_Ops'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D25" s="9">
         <f>COUNT('21_Ops'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E25" s="9" t="n"/>
       <c r="F25" s="9" t="n"/>
@@ -7608,13 +8163,13 @@
           <t>22. Roadmap &amp; Recommendations</t>
         </is>
       </c>
-      <c r="C26" s="12" t="str">
+      <c r="C26" s="12">
         <f>IFERROR(AVERAGE('22_Roadmap'!J5:J200),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D26" s="9">
         <f>COUNT('22_Roadmap'!J5:J200)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="E26" s="9" t="n"/>
       <c r="F26" s="9" t="n"/>
@@ -7626,9 +8181,9 @@
           <t>OVERALL PLATFORM MATURITY</t>
         </is>
       </c>
-      <c r="C27" s="15" t="str">
+      <c r="C27" s="15">
         <f>IFERROR(AVERAGE(C5:C26),"-")</f>
-        <v>-</v>
+        <v/>
       </c>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>

</xml_diff>